<commit_message>
Flux: fix SB attribution — sunglasses campaign spend no longer inflates strap TACOS
Campaign-intent-based attribution in load_sb(): when sunglasses SB campaigns
(01020945, 01021010, etc.) drive strap purchases, the SB spend is now correctly
attributed to sunglasses parents instead of straps. Fixes AU misattribution
affecting 38 rows / $629 AUD. All 5 markets regenerated.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/flux/20260308_Flux_CA_Feb-Mar_2026.xlsx
+++ b/flux/20260308_Flux_CA_Feb-Mar_2026.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="📊 5W Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="📋 Weekly Raw Data" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="🔍 Child ASIN Detail" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="📈 WoW Change" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="🎯 SB Attribution" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="🎯 產品象限" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="✅ 行動方案" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="📊 5W Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="📋 Weekly Raw Data" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="🔍 Child ASIN Detail" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="📈 WoW Change" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="🎯 SB Attribution" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="🎯 產品象限" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="✅ 行動方案" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>